<commit_message>
Corrida | SFE-EXE | 2026-04-15 09:36:41.176413
</commit_message>
<xml_diff>
--- a/indicadores/SFE-EXE_out.xlsx
+++ b/indicadores/SFE-EXE_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">16/03/2026</t>
+    <t xml:space="preserve">15/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">arodriguez</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1940,7 +1940,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.387434325681778</v>
+        <v>0.38452904465032</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1998,7 +1998,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.141866064600518</v>
+        <v>0.139922885421012</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2068,7 +2068,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00586626545017277</v>
+        <v>0.00533535227318323</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2098,7 +2098,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.444995674642143</v>
+        <v>0.475246238292817</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -22403,7 +22403,7 @@
         <v>445</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.270256652229731</v>
+        <v>0.269676865605464</v>
       </c>
     </row>
     <row r="6">
@@ -22411,7 +22411,7 @@
         <v>446</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.322063081548359</v>
+        <v>0.321507805845902</v>
       </c>
     </row>
     <row r="7">
@@ -22419,7 +22419,7 @@
         <v>447</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.341948880793818</v>
+        <v>0.342630268950282</v>
       </c>
     </row>
     <row r="8">
@@ -22427,7 +22427,7 @@
         <v>448</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.332717068758387</v>
+        <v>0.333782366443654</v>
       </c>
     </row>
     <row r="9">
@@ -22435,7 +22435,7 @@
         <v>449</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.313895531522324</v>
+        <v>0.314890320769352</v>
       </c>
     </row>
     <row r="10">
@@ -22443,7 +22443,7 @@
         <v>450</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.317161644409767</v>
+        <v>0.317141390030131</v>
       </c>
     </row>
     <row r="11">
@@ -22451,7 +22451,7 @@
         <v>451</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.343252721478844</v>
+        <v>0.342534415844233</v>
       </c>
     </row>
     <row r="12">
@@ -22459,7 +22459,7 @@
         <v>452</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.38070810390781</v>
+        <v>0.378906855815425</v>
       </c>
     </row>
     <row r="13">
@@ -22467,7 +22467,7 @@
         <v>453</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.387434325681778</v>
+        <v>0.38452904465032</v>
       </c>
     </row>
     <row r="14">
@@ -22475,7 +22475,7 @@
         <v>454</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.376651117880351</v>
+        <v>0.374062675792456</v>
       </c>
     </row>
     <row r="15">
@@ -22483,7 +22483,7 @@
         <v>455</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.300618523775283</v>
+        <v>0.299931877241675</v>
       </c>
     </row>
     <row r="16">
@@ -22491,7 +22491,7 @@
         <v>456</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.214962936604364</v>
+        <v>0.215002405260721</v>
       </c>
     </row>
     <row r="17">
@@ -22499,7 +22499,7 @@
         <v>457</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.0923979146026854</v>
+        <v>0.0932734085686329</v>
       </c>
     </row>
     <row r="18">
@@ -22507,7 +22507,7 @@
         <v>458</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>-0.00741953245521149</v>
+        <v>-0.00624425729604784</v>
       </c>
     </row>
     <row r="19">
@@ -22515,7 +22515,7 @@
         <v>459</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>-0.107946410544758</v>
+        <v>-0.106879468410573</v>
       </c>
     </row>
     <row r="20">
@@ -22523,7 +22523,7 @@
         <v>460</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>-0.160703140097431</v>
+        <v>-0.160419784707846</v>
       </c>
     </row>
     <row r="21">
@@ -22531,7 +22531,7 @@
         <v>461</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.201083882611666</v>
+        <v>-0.201585400867189</v>
       </c>
     </row>
     <row r="22">
@@ -22539,7 +22539,7 @@
         <v>462</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.225354629142514</v>
+        <v>-0.226188024682012</v>
       </c>
     </row>
     <row r="23">
@@ -22547,7 +22547,7 @@
         <v>463</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.246435576965234</v>
+        <v>-0.247878135936144</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-EXE | 2026-06-17 11:35:38.312921
</commit_message>
<xml_diff>
--- a/indicadores/SFE-EXE_out.xlsx
+++ b/indicadores/SFE-EXE_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="466">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Expectativas empresarias para tomar personal en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Expectativas empresarias para tomar personal</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">16/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1908,9 +1914,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1921,7 +1931,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1935,7 +1945,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -1951,7 +1961,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1979,7 +1989,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1993,7 +2003,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2021,7 +2031,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2035,7 +2045,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2049,7 +2059,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2063,7 +2073,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2079,7 +2089,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2093,7 +2103,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2241,10 +2251,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2257,10 +2267,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2284,66 +2294,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>247.069769787897</v>
@@ -2396,7 +2406,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>93.8156716191868</v>
@@ -2453,7 +2463,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>148.450502880218</v>
@@ -2510,7 +2520,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>80.9575630186777</v>
@@ -2567,7 +2577,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>130.255066181385</v>
@@ -2624,7 +2634,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>169.43590653954</v>
@@ -2681,7 +2691,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>178.509364306692</v>
@@ -2738,7 +2748,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>191.367472907201</v>
@@ -2795,7 +2805,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>224.82281585079</v>
@@ -2852,7 +2862,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>270.651055749586</v>
@@ -2909,7 +2919,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>246.438994649004</v>
@@ -2966,7 +2976,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>211.455235022713</v>
@@ -3023,7 +3033,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>212.886609376355</v>
@@ -3082,7 +3092,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>183.895213569546</v>
@@ -3141,7 +3151,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>147.722685412265</v>
@@ -3200,7 +3210,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>111.574417837249</v>
@@ -3259,7 +3269,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>110.749558040235</v>
@@ -3318,7 +3328,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>230.766658505742</v>
@@ -3377,7 +3387,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>252.698224873403</v>
@@ -3436,7 +3446,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>149.178320348172</v>
@@ -3495,7 +3505,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>108.226457484663</v>
@@ -3554,7 +3564,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>146.121486982768</v>
@@ -3613,7 +3623,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>145.442190679344</v>
@@ -3672,7 +3682,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>54.2951831093199</v>
@@ -3731,7 +3741,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>81.5398169930403</v>
@@ -3790,7 +3800,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>135.83500010236</v>
@@ -3849,7 +3859,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>63.878113104039</v>
@@ -3908,7 +3918,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>48.2057769607769</v>
@@ -3967,7 +3977,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>84.9605590924211</v>
@@ -4026,7 +4036,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>40.7092570408574</v>
@@ -4085,7 +4095,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>156.747622014887</v>
@@ -4144,7 +4154,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>44.1299991402381</v>
@@ -4203,7 +4213,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>81.5155564107752</v>
@@ -4262,7 +4272,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>166.087946186954</v>
@@ -4321,7 +4331,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>194.303003361279</v>
@@ -4380,7 +4390,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>169.169040134624</v>
@@ -4439,7 +4449,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>229.092678329449</v>
@@ -4498,7 +4508,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>265.653375802973</v>
@@ -4557,7 +4567,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>275.333348126752</v>
@@ -4616,7 +4626,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>175.404009776757</v>
@@ -4675,7 +4685,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>204.589490241687</v>
@@ -4734,7 +4744,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>201.581178040813</v>
@@ -4793,7 +4803,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>364.685072609159</v>
@@ -4852,7 +4862,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>328.973495514914</v>
@@ -4911,7 +4921,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>293.237657838405</v>
@@ -4970,7 +4980,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>275.187784633162</v>
@@ -5029,7 +5039,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>321.307151519139</v>
@@ -5088,7 +5098,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>269.074117902354</v>
@@ -5147,7 +5157,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>335.620895055555</v>
@@ -5206,7 +5216,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>248.74374996419</v>
@@ -5265,7 +5275,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>242.678604397912</v>
@@ -5324,7 +5334,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>141.560497516927</v>
@@ -5383,7 +5393,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>214.730413628503</v>
@@ -5442,7 +5452,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>215.967703324024</v>
@@ -5501,7 +5511,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>194.4970880194</v>
@@ -5560,7 +5570,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>322.64148354372</v>
@@ -5619,7 +5629,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>205.584174114556</v>
@@ -5678,7 +5688,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>284.989059868267</v>
@@ -5737,7 +5747,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>201.265790471366</v>
@@ -5796,7 +5806,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>186.321271796058</v>
@@ -5855,7 +5865,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>196.898885663646</v>
@@ -5914,7 +5924,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>367.401997373313</v>
@@ -5973,7 +5983,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>262.899925174747</v>
@@ -6032,7 +6042,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>193.727117918782</v>
@@ -6091,7 +6101,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>280.569189395315</v>
@@ -6150,7 +6160,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>193.989423412604</v>
@@ -6209,7 +6219,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>275.234618566318</v>
@@ -6268,7 +6278,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>370.887172994493</v>
@@ -6327,7 +6337,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>253.589017398808</v>
@@ -6386,7 +6396,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>245.803432717477</v>
@@ -6445,7 +6455,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>394.667426374663</v>
@@ -6504,7 +6514,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>191.794236506417</v>
@@ -6563,7 +6573,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>278.006851049129</v>
@@ -6622,7 +6632,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>226.437592765675</v>
@@ -6681,7 +6691,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>317.156525694319</v>
@@ -6740,7 +6750,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>286.648107516028</v>
@@ -6799,7 +6809,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>313.839643399136</v>
@@ -6858,7 +6868,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>203.194541298152</v>
@@ -6917,7 +6927,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>313.462154244749</v>
@@ -6976,7 +6986,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>217.061446829708</v>
@@ -7035,7 +7045,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>237.275428918489</v>
@@ -7094,7 +7104,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>141.192907719785</v>
@@ -7153,7 +7163,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>256.850229162607</v>
@@ -7212,7 +7222,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>196.668021855268</v>
@@ -7271,7 +7281,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>286.037127923111</v>
@@ -7330,7 +7340,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>167.315394797293</v>
@@ -7389,7 +7399,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>280.33737181269</v>
@@ -7448,7 +7458,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>229.231240071724</v>
@@ -7507,7 +7517,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>93.1741403259203</v>
@@ -7566,7 +7576,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>127.710239757245</v>
@@ -7625,7 +7635,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>132.279682651078</v>
@@ -7684,7 +7694,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>99.6587171938425</v>
@@ -7743,7 +7753,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>80.3113458922652</v>
@@ -7802,7 +7812,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>27.2568767468919</v>
@@ -7861,7 +7871,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>93.9788411895276</v>
@@ -7920,7 +7930,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>94.679516585481</v>
@@ -7979,7 +7989,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>135.399205282922</v>
@@ -8038,7 +8048,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>100.337482914543</v>
@@ -8097,7 +8107,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>156.9898427577</v>
@@ -8156,7 +8166,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>167.204646384016</v>
@@ -8215,7 +8225,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>119.760052894567</v>
@@ -8274,7 +8284,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>103.348482324159</v>
@@ -8333,7 +8343,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>122.931036454072</v>
@@ -8392,7 +8402,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>97.3742291274146</v>
@@ -8451,7 +8461,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>44.1011276756101</v>
@@ -8510,7 +8520,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>89.335412949483</v>
@@ -8569,7 +8579,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>64.6511849663361</v>
@@ -8628,7 +8638,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>65.7341186563818</v>
@@ -8687,7 +8697,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>53.5078892176103</v>
@@ -8746,7 +8756,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>130.453437809778</v>
@@ -8805,7 +8815,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>71.231112744691</v>
@@ -8864,7 +8874,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>163.169167825247</v>
@@ -8923,7 +8933,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>76.792672448185</v>
@@ -8982,7 +8992,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>82.0709897119553</v>
@@ -9041,7 +9051,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>89.0270542999881</v>
@@ -9100,7 +9110,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>116.894785300227</v>
@@ -9159,7 +9169,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>110.139831748154</v>
@@ -9218,7 +9228,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>116.155566993463</v>
@@ -9277,7 +9287,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>103.529723448101</v>
@@ -9336,7 +9346,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>87.0277684526003</v>
@@ -9395,7 +9405,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>92.2764803847932</v>
@@ -9454,7 +9464,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>94.9032047969642</v>
@@ -9513,7 +9523,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>83.8335771078799</v>
@@ -9572,7 +9582,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>58.3956324021368</v>
@@ -9631,7 +9641,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>125.725311396317</v>
@@ -9690,7 +9700,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>122.18966606755</v>
@@ -9749,7 +9759,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>115.482258972764</v>
@@ -9808,7 +9818,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>204.14129764949</v>
@@ -9867,7 +9877,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>161.526841972502</v>
@@ -9926,7 +9936,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>157.242455444863</v>
@@ -9985,7 +9995,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>194.344527958037</v>
@@ -10044,7 +10054,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>151.475195762281</v>
@@ -10103,7 +10113,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>174.135194632885</v>
@@ -10162,7 +10172,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>166.186189950582</v>
@@ -10221,7 +10231,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>204.657887287429</v>
@@ -10280,7 +10290,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>200.803307254126</v>
@@ -10339,7 +10349,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>188.279353302567</v>
@@ -10398,7 +10408,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>193.440156845696</v>
@@ -10457,7 +10467,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>161.207969282415</v>
@@ -10516,7 +10526,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>162.700475016514</v>
@@ -10575,7 +10585,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>215.771615861669</v>
@@ -10634,7 +10644,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>172.873621753923</v>
@@ -10693,7 +10703,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>220.987922404899</v>
@@ -10752,7 +10762,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>112.01812258123</v>
@@ -10811,7 +10821,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>177.965508330922</v>
@@ -10870,7 +10880,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>238.220808167539</v>
@@ -10929,7 +10939,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>242.443695368022</v>
@@ -10988,7 +10998,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>164.160405848827</v>
@@ -11047,7 +11057,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>162.257405615006</v>
@@ -11106,7 +11116,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>179.481530934726</v>
@@ -11165,7 +11175,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>121.578489697434</v>
@@ -11224,7 +11234,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>168.805814368969</v>
@@ -11283,7 +11293,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>89.7090185320252</v>
@@ -11342,7 +11352,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>173.033189209489</v>
@@ -11401,7 +11411,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>164.196357764322</v>
@@ -11460,7 +11470,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>188.974636885313</v>
@@ -11519,7 +11529,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>133.752093620127</v>
@@ -11578,7 +11588,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>193.131287203558</v>
@@ -11637,7 +11647,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>70.6899415718965</v>
@@ -11696,7 +11706,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>161.707047207902</v>
@@ -11755,7 +11765,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>57.9489935393838</v>
@@ -11814,7 +11824,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>128.666330994356</v>
@@ -11873,7 +11883,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>135.429491393959</v>
@@ -11932,7 +11942,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>104.606222993769</v>
@@ -11991,7 +12001,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>138.08974979944</v>
@@ -12050,7 +12060,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>186.245378798393</v>
@@ -12109,7 +12119,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>267.709460390033</v>
@@ -12168,7 +12178,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>144.896736367052</v>
@@ -12227,7 +12237,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>186.007341794349</v>
@@ -12286,7 +12296,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>136.145110725847</v>
@@ -12345,7 +12355,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>156.352921468739</v>
@@ -12404,7 +12414,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>117.941456722079</v>
@@ -12463,7 +12473,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>187.884906951202</v>
@@ -12522,7 +12532,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>162.927618431054</v>
@@ -12581,7 +12591,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>187.509160280554</v>
@@ -12640,7 +12650,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>188.942275283815</v>
@@ -12699,7 +12709,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>135.494750151296</v>
@@ -12758,7 +12768,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>312.795594841843</v>
@@ -12817,7 +12827,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>270.706989644081</v>
@@ -12876,7 +12886,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>239.391292105928</v>
@@ -12935,7 +12945,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>233.900806051599</v>
@@ -12994,7 +13004,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>154.079032066614</v>
@@ -13053,7 +13063,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>285.668779204106</v>
@@ -13112,7 +13122,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>238.287019244052</v>
@@ -13171,7 +13181,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>257.298092624207</v>
@@ -13230,7 +13240,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>297.485583956916</v>
@@ -13289,7 +13299,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>237.604860853378</v>
@@ -13348,7 +13358,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>237.522785218107</v>
@@ -13407,7 +13417,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>176.025437656223</v>
@@ -13466,7 +13476,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>190.901346899675</v>
@@ -13525,7 +13535,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>168.737741592496</v>
@@ -13584,7 +13594,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>148.107833345183</v>
@@ -13643,7 +13653,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>184.051525673858</v>
@@ -13702,7 +13712,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>177.927484263412</v>
@@ -13761,7 +13771,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>257.642909177481</v>
@@ -13820,7 +13830,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>183.87588154784</v>
@@ -13879,7 +13889,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>146.372734690327</v>
@@ -13938,7 +13948,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>211.604213159069</v>
@@ -13997,7 +14007,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>184.108729520365</v>
@@ -14056,7 +14066,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>194.268346678807</v>
@@ -14115,7 +14125,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>207.342519965556</v>
@@ -14174,7 +14184,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>163.493316304785</v>
@@ -14233,7 +14243,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>185.273858047181</v>
@@ -14292,7 +14302,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>265.397378683214</v>
@@ -14351,7 +14361,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>244.345405341253</v>
@@ -14410,7 +14420,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>296.029242273605</v>
@@ -14469,7 +14479,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>239.925817705339</v>
@@ -14528,7 +14538,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>201.359389930039</v>
@@ -14587,7 +14597,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>223.86489801906</v>
@@ -14646,7 +14656,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>262.104663454742</v>
@@ -14705,7 +14715,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>274.554368923913</v>
@@ -14764,7 +14774,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>223.612544472782</v>
@@ -14823,7 +14833,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>364.014569484427</v>
@@ -14882,7 +14892,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>387.847914446044</v>
@@ -14941,7 +14951,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>294.39073861239</v>
@@ -15000,7 +15010,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>261.132619577915</v>
@@ -15059,7 +15069,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>185.828648306808</v>
@@ -15118,7 +15128,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>484.613690414862</v>
@@ -15177,7 +15187,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>227.689267568603</v>
@@ -15236,7 +15246,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>197.526562789702</v>
@@ -15295,7 +15305,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>134.28238166621</v>
@@ -15354,7 +15364,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>107.519466016434</v>
@@ -15413,7 +15423,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>166.832562052552</v>
@@ -15472,7 +15482,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>101.653528657267</v>
@@ -15531,7 +15541,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>185.148318053719</v>
@@ -15590,7 +15600,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>202.067069846618</v>
@@ -15649,7 +15659,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>139.608070570567</v>
@@ -15708,7 +15718,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>224.630670806339</v>
@@ -15767,7 +15777,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>144.370934653429</v>
@@ -15826,7 +15836,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>170.115996264876</v>
@@ -15885,7 +15895,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>166.167917574346</v>
@@ -15944,7 +15954,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>158.33678789649</v>
@@ -16003,7 +16013,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>120.832231548491</v>
@@ -16062,7 +16072,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>175.45142159081</v>
@@ -16121,7 +16131,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>145.99109844859</v>
@@ -16180,7 +16190,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>115.462217722038</v>
@@ -16239,7 +16249,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>124.019322346907</v>
@@ -16298,7 +16308,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>156.808916822915</v>
@@ -16357,7 +16367,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>116.220385013042</v>
@@ -16416,7 +16426,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>217.256361410783</v>
@@ -16475,7 +16485,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>189.868253583983</v>
@@ -16534,7 +16544,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>174.03231562615</v>
@@ -16593,7 +16603,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>20.5337192102181</v>
@@ -16652,7 +16662,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>19.9511243823657</v>
@@ -16711,7 +16721,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>63.2219779430978</v>
@@ -16770,7 +16780,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>64.8322024787023</v>
@@ -16829,7 +16839,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>154.125898923595</v>
@@ -16888,7 +16898,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>87.6199021354032</v>
@@ -16947,7 +16957,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>144.151859010319</v>
@@ -17006,7 +17016,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>143.592331900807</v>
@@ -17065,7 +17075,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>189.964597667143</v>
@@ -17124,7 +17134,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>151.62795088673</v>
@@ -17183,7 +17193,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>134.232516288434</v>
@@ -17242,7 +17252,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>195.617215680333</v>
@@ -17301,7 +17311,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>170.460095224338</v>
@@ -17360,7 +17370,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>202.500958197938</v>
@@ -17419,7 +17429,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>116.237018770521</v>
@@ -17478,7 +17488,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>199.962824090673</v>
@@ -17537,7 +17547,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>175.709748378356</v>
@@ -17596,7 +17606,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>229.454485657326</v>
@@ -17655,7 +17665,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>171.041330724924</v>
@@ -17714,7 +17724,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>285.481725065735</v>
@@ -17773,7 +17783,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>191.355455333427</v>
@@ -17832,7 +17842,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>236.152366609554</v>
@@ -17891,7 +17901,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>253.588407105968</v>
@@ -17950,7 +17960,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>216.057665152524</v>
@@ -18009,7 +18019,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>216.303266566422</v>
@@ -18068,7 +18078,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>201.242627976442</v>
@@ -18127,7 +18137,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>281.498881116617</v>
@@ -18186,7 +18196,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>195.719764458494</v>
@@ -18245,7 +18255,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>263.265458640722</v>
@@ -18304,7 +18314,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>277.193954613936</v>
@@ -18363,7 +18373,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>174.578075982755</v>
@@ -18422,7 +18432,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>248.425721029365</v>
@@ -18481,7 +18491,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>162.710700421563</v>
@@ -18540,7 +18550,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>174.812455189884</v>
@@ -18599,7 +18609,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>198.887170579405</v>
@@ -18658,7 +18668,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>160.39106393029</v>
@@ -18717,7 +18727,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>238.542996727991</v>
@@ -18776,7 +18786,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>205.927555166975</v>
@@ -18835,7 +18845,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>173.710477075859</v>
@@ -18894,7 +18904,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>147.790786391871</v>
@@ -18953,7 +18963,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>170.600156221783</v>
@@ -19012,7 +19022,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>152.987225887006</v>
@@ -19071,7 +19081,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>104.411822516331</v>
@@ -19130,7 +19140,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>102.85233595093</v>
@@ -19189,7 +19199,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>91.6102275319021</v>
@@ -19248,7 +19258,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>125.406327276909</v>
@@ -19307,7 +19317,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>73.8861790230734</v>
@@ -19366,7 +19376,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>83.8405436348305</v>
@@ -19425,7 +19435,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>141.662781747654</v>
@@ -19484,7 +19494,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>120.304690164102</v>
@@ -19543,7 +19553,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>136.752168263315</v>
@@ -19602,7 +19612,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>128.568394032186</v>
@@ -19661,7 +19671,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>122.004014069333</v>
@@ -19720,7 +19730,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>119.104776663859</v>
@@ -19779,7 +19789,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>113.334308087044</v>
@@ -19838,7 +19848,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>135.965464245969</v>
@@ -19897,7 +19907,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>208.942436873937</v>
@@ -19956,7 +19966,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>176.976355117024</v>
@@ -20015,7 +20025,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>202.465152704476</v>
@@ -20074,7 +20084,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>138.963997861076</v>
@@ -20133,7 +20143,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>108.073876840728</v>
@@ -20192,7 +20202,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>141.793585256653</v>
@@ -20251,7 +20261,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>103.732832154247</v>
@@ -20310,7 +20320,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>113.505525754463</v>
@@ -20369,7 +20379,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>143.725601776603</v>
@@ -20428,7 +20438,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>82.0948908907033</v>
@@ -20487,7 +20497,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>142.182300091488</v>
@@ -20546,7 +20556,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>127.597459145387</v>
@@ -20605,7 +20615,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>220.970576928642</v>
@@ -20664,7 +20674,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>179.435429580954</v>
@@ -20723,7 +20733,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>129.820528423085</v>
@@ -20782,7 +20792,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>112.131666482356</v>
@@ -20841,7 +20851,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>102.237841776509</v>
@@ -20900,7 +20910,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>106.236741579406</v>
@@ -20959,7 +20969,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2"/>
       <c r="C318" s="3" t="n">
@@ -20992,7 +21002,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2"/>
       <c r="C319" s="3" t="n">
@@ -21025,7 +21035,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2"/>
       <c r="C320" s="3" t="n">
@@ -21058,7 +21068,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2"/>
       <c r="C321" s="3" t="n">
@@ -21091,7 +21101,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2"/>
       <c r="C322" s="3" t="n">
@@ -21124,7 +21134,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2"/>
       <c r="C323" s="3" t="n">
@@ -21157,7 +21167,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2"/>
       <c r="C324" s="3" t="n">
@@ -21190,7 +21200,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2"/>
       <c r="C325" s="3" t="n">
@@ -21223,7 +21233,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2"/>
       <c r="C326" s="3" t="n">
@@ -21256,7 +21266,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2"/>
       <c r="C327" s="3" t="n">
@@ -21289,7 +21299,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2"/>
       <c r="C328" s="3" t="n">
@@ -21322,7 +21332,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2"/>
       <c r="C329" s="3" t="n">
@@ -21355,7 +21365,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2"/>
       <c r="C330" s="3"/>
@@ -21378,7 +21388,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2"/>
       <c r="C331" s="3"/>
@@ -21401,7 +21411,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2"/>
       <c r="C332" s="3"/>
@@ -21424,7 +21434,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2"/>
       <c r="C333" s="3"/>
@@ -21447,7 +21457,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2"/>
       <c r="C334" s="3"/>
@@ -21470,7 +21480,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2"/>
       <c r="C335" s="3"/>
@@ -21493,7 +21503,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2"/>
       <c r="C336" s="3"/>
@@ -21516,7 +21526,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2"/>
       <c r="C337" s="3"/>
@@ -21539,7 +21549,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2"/>
       <c r="C338" s="3"/>
@@ -21562,7 +21572,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2"/>
       <c r="C339" s="3"/>
@@ -21585,7 +21595,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2"/>
       <c r="C340" s="3"/>
@@ -21608,7 +21618,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2"/>
       <c r="C341" s="3"/>
@@ -21631,7 +21641,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2"/>
       <c r="C342" s="3"/>
@@ -21654,7 +21664,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2"/>
       <c r="C343" s="3"/>
@@ -21677,7 +21687,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2"/>
       <c r="C344" s="3"/>
@@ -21700,7 +21710,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2"/>
       <c r="C345" s="3"/>
@@ -21723,7 +21733,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2"/>
       <c r="C346" s="3"/>
@@ -21746,7 +21756,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2"/>
       <c r="C347" s="3"/>
@@ -21769,7 +21779,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2"/>
       <c r="C348" s="3"/>
@@ -21792,7 +21802,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2"/>
       <c r="C349" s="3"/>
@@ -21815,7 +21825,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2"/>
       <c r="C350" s="3"/>
@@ -21838,7 +21848,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2"/>
       <c r="C351" s="3"/>
@@ -21861,7 +21871,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2"/>
       <c r="C352" s="3"/>
@@ -21884,7 +21894,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2"/>
       <c r="C353" s="3"/>
@@ -21907,7 +21917,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2"/>
       <c r="C354" s="3"/>
@@ -21930,7 +21940,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2"/>
       <c r="C355" s="3"/>
@@ -21953,7 +21963,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2"/>
       <c r="C356" s="3"/>
@@ -21976,7 +21986,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2"/>
       <c r="C357" s="3"/>
@@ -21999,7 +22009,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2"/>
       <c r="C358" s="3"/>
@@ -22022,7 +22032,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2"/>
       <c r="C359" s="3"/>
@@ -22045,7 +22055,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2"/>
       <c r="C360" s="3"/>
@@ -22068,7 +22078,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2"/>
       <c r="C361" s="3"/>
@@ -22091,7 +22101,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2"/>
       <c r="C362" s="3"/>
@@ -22114,7 +22124,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2"/>
       <c r="C363" s="3"/>
@@ -22137,7 +22147,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2"/>
       <c r="C364" s="3"/>
@@ -22160,7 +22170,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2"/>
       <c r="C365" s="3"/>
@@ -22183,7 +22193,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2"/>
       <c r="C366" s="3"/>
@@ -22206,7 +22216,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2"/>
       <c r="C367" s="3"/>
@@ -22229,7 +22239,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2"/>
       <c r="C368" s="3"/>
@@ -22252,7 +22262,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2"/>
       <c r="C369" s="3"/>
@@ -22275,7 +22285,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2"/>
       <c r="C370" s="3"/>
@@ -22298,7 +22308,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2"/>
       <c r="C371" s="3"/>
@@ -22321,7 +22331,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2"/>
       <c r="C372" s="3"/>
@@ -22344,7 +22354,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2"/>
       <c r="C373" s="3"/>
@@ -22378,97 +22388,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
   </sheetData>
@@ -22492,7 +22502,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -22502,13 +22512,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.27450604325712</v>
@@ -22516,7 +22526,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.322536186223231</v>
@@ -22524,7 +22534,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.344276767496809</v>
@@ -22532,7 +22542,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.337839297703177</v>
@@ -22540,7 +22550,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.320276077642269</v>
@@ -22548,7 +22558,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.324600566971095</v>
@@ -22556,7 +22566,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.349265467210488</v>
@@ -22564,7 +22574,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.385421483420625</v>
@@ -22572,7 +22582,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.388734632550379</v>
@@ -22580,7 +22590,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.374458639412818</v>
@@ -22588,7 +22598,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.298412575062608</v>
@@ -22596,7 +22606,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.214544137098633</v>
@@ -22604,7 +22614,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.0980532621207997</v>
@@ -22612,7 +22622,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.00680443546305185</v>
@@ -22620,7 +22630,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>-0.0884512017744036</v>
@@ -22628,7 +22638,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.145484621102778</v>
@@ -22636,7 +22646,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.195579283351881</v>
@@ -22644,7 +22654,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.227306656304438</v>
@@ -22652,7 +22662,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.259332823657891</v>

</xml_diff>

<commit_message>
Corrida | SFE-EXE | 2026-07-15 10:56:55.601173
</commit_message>
<xml_diff>
--- a/indicadores/SFE-EXE_out.xlsx
+++ b/indicadores/SFE-EXE_out.xlsx
@@ -22729,237 +22729,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{114833E3-ABDA-4757-BF2E-CC3EAF6CF8C7}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{482F8CB7-2A4B-46E1-A716-1A656DA3900D}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6178E0FE-19C8-4CFD-905A-CC5431EFEA01}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-EXE | 2026-08-25 13:08:35.185151
</commit_message>
<xml_diff>
--- a/indicadores/SFE-EXE_out.xlsx
+++ b/indicadores/SFE-EXE_out.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Unidad de medida</t>
   </si>
   <si>
-    <t xml:space="preserve">Índice base 2009=100</t>
+    <t xml:space="preserve">Índice base 2010=100</t>
   </si>
   <si>
     <t xml:space="preserve">Ajuste estacional</t>
@@ -22765,237 +22765,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB534F58-E77E-4A6E-90FE-D1D379537D3D}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE366F25-0251-428E-B2FD-172BCF4C7CAF}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6DA22A1E-C379-4C29-A714-DDDE4B113977}"/>
 </file>
</xml_diff>